<commit_message>
Sync from terminal run 2026-10-06-0647
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Animal_Welfare.xlsx
+++ b/results/auto_Cape_Town_Animal_Welfare.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -37,22 +37,16 @@
     <t>Sent</t>
   </si>
   <si>
-    <t>Cape of Good Hope SPCA</t>
-  </si>
-  <si>
-    <t>TEARS Animal Rescue</t>
-  </si>
-  <si>
-    <t>Animal Rescue Organisation ARO</t>
-  </si>
-  <si>
-    <t>African Bird of Prey Sanctuary</t>
-  </si>
-  <si>
-    <t>Cheetah Outreach</t>
-  </si>
-  <si>
-    <t>Panthera Africa</t>
+    <t>African Tails</t>
+  </si>
+  <si>
+    <t>Animal Anti-Cruelty League</t>
+  </si>
+  <si>
+    <t>Animal Lifeline</t>
+  </si>
+  <si>
+    <t>Animal Rescue Organisation</t>
   </si>
   <si>
     <t>Animal Welfare</t>
@@ -61,22 +55,16 @@
     <t>Cape Town</t>
   </si>
   <si>
-    <t>info@capespca.co.za</t>
-  </si>
-  <si>
-    <t>adoptions@tears.org.za</t>
-  </si>
-  <si>
-    <t>aro@animalrescue.org.za</t>
-  </si>
-  <si>
-    <t>info@africanbirdofprey.org.za</t>
-  </si>
-  <si>
-    <t>info@cheetah.co.za</t>
-  </si>
-  <si>
-    <t>info@pantheraafrica.org</t>
+    <t>adoptions@africantails.co.za</t>
+  </si>
+  <si>
+    <t>controlinspector@aacl-ct.co.za</t>
+  </si>
+  <si>
+    <t>hello@animallifeline.org.za</t>
+  </si>
+  <si>
+    <t>vet@animalrescue.org.za</t>
   </si>
   <si>
     <t>Yes</t>
@@ -411,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -442,16 +430,16 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -459,16 +447,16 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -476,16 +464,16 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" t="s">
         <v>17</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -493,50 +481,16 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>